<commit_message>
fix: anchor report bullets for RTL
</commit_message>
<xml_diff>
--- a/reports/דו״ח-קשרים-אחדות-יהודית.xlsx
+++ b/reports/דו״ח-קשרים-אחדות-יהודית.xlsx
@@ -22,10 +22,10 @@
     <t>טווח: כל ההיסטוריה הקיימת במערכת</t>
   </si>
   <si>
-    <t>• האפליקציה עדיין בפיילוט ראשוני, הערכה שמשקפת 75% מהקשרים והלקוחות האמיתיים</t>
-  </si>
-  <si>
-    <t>• האפליקציה עלתה לאוויר לפני כחודש וחצי</t>
+    <t>‏• האפליקציה עדיין בפיילוט ראשוני, הערכה שמשקפת 75% מהקשרים והלקוחות האמיתיים</t>
+  </si>
+  <si>
+    <t>‏• האפליקציה עלתה לאוויר לפני כחודש וחצי</t>
   </si>
   <si>
     <t>שם הפעיל</t>

</xml_diff>

<commit_message>
feat: add executive analytics to live reports
</commit_message>
<xml_diff>
--- a/reports/דו״ח-קשרים-אחדות-יהודית.xlsx
+++ b/reports/דו״ח-קשרים-אחדות-יהודית.xlsx
@@ -9,12 +9,15 @@
     <sheet sheetId="3" name="סיכום מצוות" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="סיכום ארגוני" state="visible" r:id="rId7"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'סיכום ארגוני'!$A1:$N61</definedName>
+  </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="131">
   <si>
     <t>דו״ח קשרים — אחדות יהודית</t>
   </si>
@@ -328,14 +331,92 @@
     <t>משפט סיכום</t>
   </si>
   <si>
-    <t>בכל ההיסטוריה הקיימת במערכת בוצעו בסך הכול 765 קשרים: 426 קשרים תורניים, 258 קשרים ידידותיים, 269 קשרים פרונטליים, 34 קשרי וידאו, 457 קשרים טלפוניים ו־5 אירוחי שבת.</t>
+    <t>בכל ההיסטוריה הקיימת במערכת בוצעו בסך הכול 797 קשרים: 438 קשרים תורניים, 274 קשרים ידידותיים, 276 קשרים פרונטליים, 36 קשרי וידאו, 479 קשרים טלפוניים ו־6 אירוחי שבת.</t>
+  </si>
+  <si>
+    <t>תמונת מצב מנהלים</t>
+  </si>
+  <si>
+    <t>ניתוח איכות הקשר, אופן הקשר ועומק הקשר עם הלקוחות</t>
+  </si>
+  <si>
+    <t>לקוחות פעילים בקשר</t>
+  </si>
+  <si>
+    <t>קשרים לפי איכות ואופן הקשר</t>
+  </si>
+  <si>
+    <t>תורני · פרונטלי</t>
+  </si>
+  <si>
+    <t>ידידותי · פרונטלי</t>
+  </si>
+  <si>
+    <t>תורני · וידאו</t>
+  </si>
+  <si>
+    <t>ידידותי · וידאו</t>
+  </si>
+  <si>
+    <t>תורני · טלפוני</t>
+  </si>
+  <si>
+    <t>ידידותי · טלפוני</t>
+  </si>
+  <si>
+    <t>תורני · סוגים נוספים</t>
+  </si>
+  <si>
+    <t>ידידותי · סוגים נוספים</t>
+  </si>
+  <si>
+    <t>סוגים נוספים כוללים אירוח שבת וכל סוג קשר שאינו פרונטלי, וידאו או טלפוני.</t>
+  </si>
+  <si>
+    <t>התפלגות לקוחות לפי מספר קשרים</t>
+  </si>
+  <si>
+    <t>0 קשרים</t>
+  </si>
+  <si>
+    <t>קשר אחד</t>
+  </si>
+  <si>
+    <t>2 קשרים</t>
+  </si>
+  <si>
+    <t>3–4 קשרים</t>
+  </si>
+  <si>
+    <t>5–9 קשרים</t>
+  </si>
+  <si>
+    <t>10 קשרים ומעלה</t>
+  </si>
+  <si>
+    <t>מפת עומק הקשר עם הלקוחות</t>
+  </si>
+  <si>
+    <t>קשר כללי · נתון הנהלה משוער</t>
+  </si>
+  <si>
+    <t>↓ מידע מתועד ב־CRM</t>
+  </si>
+  <si>
+    <t>קשר אישי תורני</t>
+  </si>
+  <si>
+    <t>קשר אישי ידידותי</t>
+  </si>
+  <si>
+    <t>המאגר הכללי הוא נתון הנהלה משוער. הקבוצות האישיות מחושבות מנתוני ה־CRM; קשר תורני אחד לפחות מסווג לקוח כ״אישי תורני״. 9 לקוחות פעילים טרם סווגו כאישי תורני או ידידותי.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -365,8 +446,72 @@
       <b/>
       <color rgb="FF3A249B"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF3A249B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF4F46E5"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F766E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFD97706"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF3A249B"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF211F2D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF4F46E5"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F766E"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF6B6574"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFD97706"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="FF5E5650"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -388,8 +533,33 @@
         <fgColor rgb="FFF0EFFE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4F46E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F766E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD97706"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8EAF2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -406,11 +576,80 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3A249B"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3A249B"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3A249B"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3A249B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF4F46E5"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF4F46E5"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF4F46E5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF4F46E5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF0F766E"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF0F766E"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF0F766E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF0F766E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD97706"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD97706"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD97706"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD97706"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -463,6 +702,64 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -915,13 +1212,13 @@
         <v>26</v>
       </c>
       <c r="C7" s="12">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D7" s="12">
         <v>16</v>
       </c>
       <c r="E7" s="12">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="F7" s="12">
         <v>45</v>
@@ -930,19 +1227,19 @@
         <v>0</v>
       </c>
       <c r="H7" s="12">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="I7" s="12">
         <v>0</v>
       </c>
       <c r="J7" s="12">
-        <v>993</v>
+        <v>1018</v>
       </c>
       <c r="K7" s="13">
-        <v>3.576923076923077</v>
+        <v>3.769230769230769</v>
       </c>
       <c r="L7" s="13">
-        <v>10.67741935483871</v>
+        <v>10.387755102040817</v>
       </c>
     </row>
     <row r="8" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1143,19 +1440,19 @@
         <v>14</v>
       </c>
       <c r="C13" s="12">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D13" s="12">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E13" s="12">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F13" s="12">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G13" s="12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H13" s="12">
         <v>30</v>
@@ -1164,13 +1461,13 @@
         <v>0</v>
       </c>
       <c r="J13" s="12">
-        <v>605</v>
+        <v>626</v>
       </c>
       <c r="K13" s="13">
-        <v>3.142857142857143</v>
+        <v>3.2857142857142856</v>
       </c>
       <c r="L13" s="13">
-        <v>13.75</v>
+        <v>13.608695652173912</v>
       </c>
     </row>
     <row r="14" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1523,10 +1820,10 @@
         <v>14</v>
       </c>
       <c r="C23" s="12">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D23" s="12">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E23" s="12">
         <v>5</v>
@@ -1538,19 +1835,19 @@
         <v>5</v>
       </c>
       <c r="H23" s="12">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I23" s="12">
         <v>0</v>
       </c>
       <c r="J23" s="12">
-        <v>531</v>
+        <v>547</v>
       </c>
       <c r="K23" s="13">
-        <v>2.7142857142857144</v>
+        <v>2.7857142857142856</v>
       </c>
       <c r="L23" s="13">
-        <v>13.973684210526315</v>
+        <v>14.025641025641026</v>
       </c>
     </row>
     <row r="24" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1558,19 +1855,19 @@
         <v>33</v>
       </c>
       <c r="B24" s="12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C24" s="12">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D24" s="12">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E24" s="12">
         <v>4</v>
       </c>
       <c r="F24" s="12">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G24" s="12">
         <v>7</v>
@@ -1582,10 +1879,10 @@
         <v>0</v>
       </c>
       <c r="J24" s="12">
-        <v>512</v>
+        <v>528</v>
       </c>
       <c r="K24" s="13">
-        <v>4</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="L24" s="13">
         <v>16</v>
@@ -1637,10 +1934,10 @@
         <v>21</v>
       </c>
       <c r="C26" s="12">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D26" s="12">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E26" s="12">
         <v>2</v>
@@ -1652,19 +1949,19 @@
         <v>0</v>
       </c>
       <c r="H26" s="12">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I26" s="12">
         <v>0</v>
       </c>
       <c r="J26" s="12">
-        <v>693</v>
+        <v>709</v>
       </c>
       <c r="K26" s="13">
-        <v>2.0952380952380953</v>
+        <v>2.142857142857143</v>
       </c>
       <c r="L26" s="13">
-        <v>15.75</v>
+        <v>15.755555555555556</v>
       </c>
     </row>
     <row r="27" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1672,22 +1969,22 @@
         <v>36</v>
       </c>
       <c r="B27" s="12">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C27" s="12">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D27" s="12">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E27" s="12">
         <v>2</v>
       </c>
       <c r="F27" s="12">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G27" s="12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H27" s="12">
         <v>14</v>
@@ -1696,13 +1993,13 @@
         <v>0</v>
       </c>
       <c r="J27" s="12">
-        <v>490</v>
+        <v>522</v>
       </c>
       <c r="K27" s="13">
-        <v>2.4615384615384617</v>
+        <v>2.4285714285714284</v>
       </c>
       <c r="L27" s="13">
-        <v>15.3125</v>
+        <v>15.352941176470589</v>
       </c>
     </row>
     <row r="28" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1713,13 +2010,13 @@
         <v>2</v>
       </c>
       <c r="C28" s="12">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D28" s="12">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E28" s="12">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F28" s="12">
         <v>2</v>
@@ -1728,19 +2025,19 @@
         <v>0</v>
       </c>
       <c r="H28" s="12">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="I28" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" s="12">
-        <v>143</v>
+        <v>294</v>
       </c>
       <c r="K28" s="13">
-        <v>5.5</v>
+        <v>10</v>
       </c>
       <c r="L28" s="13">
-        <v>13</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="29" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1748,16 +2045,16 @@
         <v>38</v>
       </c>
       <c r="B29" s="12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C29" s="12">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D29" s="12">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E29" s="12">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F29" s="12">
         <v>12</v>
@@ -1766,19 +2063,19 @@
         <v>0</v>
       </c>
       <c r="H29" s="12">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="I29" s="12">
         <v>0</v>
       </c>
       <c r="J29" s="12">
-        <v>477</v>
+        <v>497</v>
       </c>
       <c r="K29" s="13">
-        <v>6.75</v>
+        <v>6.444444444444445</v>
       </c>
       <c r="L29" s="13">
-        <v>8.833333333333334</v>
+        <v>8.568965517241379</v>
       </c>
     </row>
     <row r="30" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1789,10 +2086,10 @@
         <v>3</v>
       </c>
       <c r="C30" s="12">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D30" s="12">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E30" s="12">
         <v>18</v>
@@ -1804,19 +2101,19 @@
         <v>0</v>
       </c>
       <c r="H30" s="12">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I30" s="12">
         <v>0</v>
       </c>
       <c r="J30" s="12">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="K30" s="13">
-        <v>10.333333333333334</v>
+        <v>10.666666666666666</v>
       </c>
       <c r="L30" s="13">
-        <v>6.096774193548387</v>
+        <v>6.0625</v>
       </c>
     </row>
     <row r="31" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1941,13 +2238,13 @@
         <v>8</v>
       </c>
       <c r="C34" s="12">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D34" s="12">
         <v>6</v>
       </c>
       <c r="E34" s="12">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F34" s="12">
         <v>6</v>
@@ -1956,19 +2253,19 @@
         <v>0</v>
       </c>
       <c r="H34" s="12">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I34" s="12">
         <v>0</v>
       </c>
       <c r="J34" s="12">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="K34" s="13">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="L34" s="13">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="35" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1979,16 +2276,16 @@
         <v>10</v>
       </c>
       <c r="C35" s="12">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D35" s="12">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E35" s="12">
         <v>38</v>
       </c>
       <c r="F35" s="12">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G35" s="12">
         <v>0</v>
@@ -2000,13 +2297,13 @@
         <v>0</v>
       </c>
       <c r="J35" s="12">
-        <v>1458</v>
+        <v>1522</v>
       </c>
       <c r="K35" s="13">
-        <v>7.1</v>
+        <v>7.5</v>
       </c>
       <c r="L35" s="13">
-        <v>20.535211267605632</v>
+        <v>20.293333333333333</v>
       </c>
     </row>
     <row r="36" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -2052,7 +2349,7 @@
         <v>46</v>
       </c>
       <c r="B37" s="12">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="C37" s="12">
         <v>34</v>
@@ -2079,7 +2376,7 @@
         <v>423</v>
       </c>
       <c r="K37" s="13">
-        <v>2</v>
+        <v>1.096774193548387</v>
       </c>
       <c r="L37" s="13">
         <v>12.441176470588236</v>
@@ -2128,37 +2425,37 @@
         <v>48</v>
       </c>
       <c r="B39" s="15">
-        <v>237</v>
+        <v>254</v>
       </c>
       <c r="C39" s="15">
-        <v>765</v>
+        <v>797</v>
       </c>
       <c r="D39" s="15">
-        <v>426</v>
+        <v>438</v>
       </c>
       <c r="E39" s="15">
-        <v>258</v>
+        <v>274</v>
       </c>
       <c r="F39" s="15">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="G39" s="15">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H39" s="15">
-        <v>457</v>
+        <v>479</v>
       </c>
       <c r="I39" s="15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J39" s="15">
-        <v>10251</v>
+        <v>10638</v>
       </c>
       <c r="K39" s="16">
-        <v>3.2278481012658227</v>
+        <v>3.1377952755905514</v>
       </c>
       <c r="L39" s="16">
-        <v>13.4</v>
+        <v>13.347553324968633</v>
       </c>
     </row>
   </sheetData>
@@ -4222,11 +4519,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="110" style="17" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" style="17" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="14" width="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4241,17 +4541,41 @@
       </c>
       <c r="B2" s="19"/>
     </row>
-    <row r="3" ht="25" customHeight="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="25" customHeight="1" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="6"/>
-    </row>
-    <row r="4" ht="25" customHeight="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+    </row>
+    <row r="4" ht="25" customHeight="1" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
@@ -4266,7 +4590,7 @@
         <v>102</v>
       </c>
       <c r="B7" s="21">
-        <v>237</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4274,7 +4598,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="21">
-        <v>765</v>
+        <v>797</v>
       </c>
     </row>
     <row r="9" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4282,7 +4606,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="21">
-        <v>426</v>
+        <v>438</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4290,7 +4614,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="21">
-        <v>258</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4298,7 +4622,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="21">
-        <v>269</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4306,7 +4630,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="21">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4314,7 +4638,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="21">
-        <v>457</v>
+        <v>479</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4322,7 +4646,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="21">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4330,7 +4654,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="21">
-        <v>10251</v>
+        <v>10638</v>
       </c>
     </row>
     <row r="16" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4338,7 +4662,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="21">
-        <v>3.2278481012658227</v>
+        <v>3.1377952755905514</v>
       </c>
     </row>
     <row r="17" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4346,22 +4670,639 @@
         <v>15</v>
       </c>
       <c r="B17" s="21">
-        <v>13.4</v>
-      </c>
-    </row>
-    <row r="18" ht="54" customHeight="1" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+        <v>13.347553324968633</v>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>103</v>
       </c>
       <c r="B18" s="21" t="s">
         <v>104</v>
       </c>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+    </row>
+    <row r="21" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="22"/>
+      <c r="N21" s="22"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="23"/>
+      <c r="J22" s="23"/>
+      <c r="K22" s="23"/>
+      <c r="L22" s="23"/>
+      <c r="M22" s="23"/>
+      <c r="N22" s="23"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="28">
+        <v>199</v>
+      </c>
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="29">
+        <v>438</v>
+      </c>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="30">
+        <v>274</v>
+      </c>
+      <c r="H25" s="30"/>
+      <c r="I25" s="30"/>
+      <c r="J25" s="31">
+        <v>797</v>
+      </c>
+      <c r="K25" s="31"/>
+      <c r="L25" s="31"/>
+      <c r="M25" s="31"/>
+      <c r="N25" s="31"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="28"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="30"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="31"/>
+      <c r="M26" s="31"/>
+      <c r="N26" s="31"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="32"/>
+      <c r="L28" s="32"/>
+      <c r="M28" s="32"/>
+      <c r="N28" s="32"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="33" t="s">
+        <v>109</v>
+      </c>
+      <c r="B30" s="33"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="34">
+        <v>176</v>
+      </c>
+      <c r="E30" s="35"/>
+      <c r="F30" s="35"/>
+      <c r="G30" s="35"/>
+      <c r="H30" s="35"/>
+      <c r="I30" s="35"/>
+      <c r="J30" s="35"/>
+      <c r="K30" s="35"/>
+      <c r="L30" s="36"/>
+      <c r="M30" s="36"/>
+      <c r="N30" s="36"/>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="B31" s="33"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="37">
+        <v>21</v>
+      </c>
+      <c r="E31" s="38"/>
+      <c r="F31" s="36"/>
+      <c r="G31" s="36"/>
+      <c r="H31" s="36"/>
+      <c r="I31" s="36"/>
+      <c r="J31" s="36"/>
+      <c r="K31" s="36"/>
+      <c r="L31" s="36"/>
+      <c r="M31" s="36"/>
+      <c r="N31" s="36"/>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="33" t="s">
+        <v>111</v>
+      </c>
+      <c r="B32" s="33"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="34">
+        <v>34</v>
+      </c>
+      <c r="E32" s="35"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="36"/>
+      <c r="I32" s="36"/>
+      <c r="J32" s="36"/>
+      <c r="K32" s="36"/>
+      <c r="L32" s="36"/>
+      <c r="M32" s="36"/>
+      <c r="N32" s="36"/>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="33" t="s">
+        <v>112</v>
+      </c>
+      <c r="B33" s="33"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="37">
+        <v>2</v>
+      </c>
+      <c r="E33" s="36"/>
+      <c r="F33" s="36"/>
+      <c r="G33" s="36"/>
+      <c r="H33" s="36"/>
+      <c r="I33" s="36"/>
+      <c r="J33" s="36"/>
+      <c r="K33" s="36"/>
+      <c r="L33" s="36"/>
+      <c r="M33" s="36"/>
+      <c r="N33" s="36"/>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="B34" s="33"/>
+      <c r="C34" s="33"/>
+      <c r="D34" s="34">
+        <v>228</v>
+      </c>
+      <c r="E34" s="35"/>
+      <c r="F34" s="35"/>
+      <c r="G34" s="35"/>
+      <c r="H34" s="35"/>
+      <c r="I34" s="35"/>
+      <c r="J34" s="35"/>
+      <c r="K34" s="35"/>
+      <c r="L34" s="35"/>
+      <c r="M34" s="35"/>
+      <c r="N34" s="36"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="37">
+        <v>251</v>
+      </c>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="38"/>
+      <c r="J35" s="38"/>
+      <c r="K35" s="38"/>
+      <c r="L35" s="38"/>
+      <c r="M35" s="38"/>
+      <c r="N35" s="38"/>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="B36" s="33"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="34">
+        <v>0</v>
+      </c>
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="36"/>
+      <c r="H36" s="36"/>
+      <c r="I36" s="36"/>
+      <c r="J36" s="36"/>
+      <c r="K36" s="36"/>
+      <c r="L36" s="36"/>
+      <c r="M36" s="36"/>
+      <c r="N36" s="36"/>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="B37" s="33"/>
+      <c r="C37" s="33"/>
+      <c r="D37" s="37">
+        <v>0</v>
+      </c>
+      <c r="E37" s="36"/>
+      <c r="F37" s="36"/>
+      <c r="G37" s="36"/>
+      <c r="H37" s="36"/>
+      <c r="I37" s="36"/>
+      <c r="J37" s="36"/>
+      <c r="K37" s="36"/>
+      <c r="L37" s="36"/>
+      <c r="M37" s="36"/>
+      <c r="N37" s="36"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="B39" s="39"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="39"/>
+      <c r="E39" s="39"/>
+      <c r="F39" s="39"/>
+      <c r="G39" s="39"/>
+      <c r="H39" s="39"/>
+      <c r="I39" s="39"/>
+      <c r="J39" s="39"/>
+      <c r="K39" s="39"/>
+      <c r="L39" s="39"/>
+      <c r="M39" s="39"/>
+      <c r="N39" s="39"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A41" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="B41" s="32"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="32"/>
+      <c r="J41" s="32"/>
+      <c r="K41" s="32"/>
+      <c r="L41" s="32"/>
+      <c r="M41" s="32"/>
+      <c r="N41" s="32"/>
+    </row>
+    <row r="43" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A43" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="B43" s="33"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="40">
+        <v>55</v>
+      </c>
+      <c r="E43" s="41"/>
+      <c r="F43" s="41"/>
+      <c r="G43" s="41"/>
+      <c r="H43" s="41"/>
+      <c r="I43" s="41"/>
+      <c r="J43" s="41"/>
+      <c r="K43" s="41"/>
+      <c r="L43" s="41"/>
+      <c r="M43" s="41"/>
+      <c r="N43" s="41"/>
+    </row>
+    <row r="44" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A44" s="33" t="s">
+        <v>120</v>
+      </c>
+      <c r="B44" s="33"/>
+      <c r="C44" s="33"/>
+      <c r="D44" s="40">
+        <v>53</v>
+      </c>
+      <c r="E44" s="41"/>
+      <c r="F44" s="41"/>
+      <c r="G44" s="41"/>
+      <c r="H44" s="41"/>
+      <c r="I44" s="41"/>
+      <c r="J44" s="41"/>
+      <c r="K44" s="41"/>
+      <c r="L44" s="41"/>
+      <c r="M44" s="41"/>
+      <c r="N44" s="41"/>
+    </row>
+    <row r="45" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A45" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="B45" s="33"/>
+      <c r="C45" s="33"/>
+      <c r="D45" s="40">
+        <v>34</v>
+      </c>
+      <c r="E45" s="41"/>
+      <c r="F45" s="41"/>
+      <c r="G45" s="41"/>
+      <c r="H45" s="41"/>
+      <c r="I45" s="41"/>
+      <c r="J45" s="41"/>
+      <c r="K45" s="36"/>
+      <c r="L45" s="36"/>
+      <c r="M45" s="36"/>
+      <c r="N45" s="36"/>
+    </row>
+    <row r="46" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A46" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="B46" s="33"/>
+      <c r="C46" s="33"/>
+      <c r="D46" s="40">
+        <v>47</v>
+      </c>
+      <c r="E46" s="41"/>
+      <c r="F46" s="41"/>
+      <c r="G46" s="41"/>
+      <c r="H46" s="41"/>
+      <c r="I46" s="41"/>
+      <c r="J46" s="41"/>
+      <c r="K46" s="41"/>
+      <c r="L46" s="41"/>
+      <c r="M46" s="41"/>
+      <c r="N46" s="36"/>
+    </row>
+    <row r="47" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A47" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="B47" s="33"/>
+      <c r="C47" s="33"/>
+      <c r="D47" s="40">
+        <v>49</v>
+      </c>
+      <c r="E47" s="41"/>
+      <c r="F47" s="41"/>
+      <c r="G47" s="41"/>
+      <c r="H47" s="41"/>
+      <c r="I47" s="41"/>
+      <c r="J47" s="41"/>
+      <c r="K47" s="41"/>
+      <c r="L47" s="41"/>
+      <c r="M47" s="41"/>
+      <c r="N47" s="36"/>
+    </row>
+    <row r="48" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A48" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="B48" s="33"/>
+      <c r="C48" s="33"/>
+      <c r="D48" s="40">
+        <v>16</v>
+      </c>
+      <c r="E48" s="41"/>
+      <c r="F48" s="41"/>
+      <c r="G48" s="41"/>
+      <c r="H48" s="36"/>
+      <c r="I48" s="36"/>
+      <c r="J48" s="36"/>
+      <c r="K48" s="36"/>
+      <c r="L48" s="36"/>
+      <c r="M48" s="36"/>
+      <c r="N48" s="36"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A51" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="B51" s="22"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="22"/>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="22"/>
+      <c r="H51" s="22"/>
+      <c r="I51" s="22"/>
+      <c r="J51" s="22"/>
+      <c r="K51" s="22"/>
+      <c r="L51" s="22"/>
+      <c r="M51" s="22"/>
+      <c r="N51" s="22"/>
+    </row>
+    <row r="53" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C53" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="D53" s="24"/>
+      <c r="E53" s="24"/>
+      <c r="F53" s="24"/>
+      <c r="G53" s="24"/>
+      <c r="H53" s="24"/>
+      <c r="I53" s="24"/>
+      <c r="J53" s="24"/>
+      <c r="K53" s="24"/>
+      <c r="L53" s="24"/>
+    </row>
+    <row r="54" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C54" s="28">
+        <v>850</v>
+      </c>
+      <c r="D54" s="28"/>
+      <c r="E54" s="28"/>
+      <c r="F54" s="28"/>
+      <c r="G54" s="28"/>
+      <c r="H54" s="28"/>
+      <c r="I54" s="28"/>
+      <c r="J54" s="28"/>
+      <c r="K54" s="28"/>
+      <c r="L54" s="28"/>
+    </row>
+    <row r="55" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C55" s="28"/>
+      <c r="D55" s="28"/>
+      <c r="E55" s="28"/>
+      <c r="F55" s="28"/>
+      <c r="G55" s="28"/>
+      <c r="H55" s="28"/>
+      <c r="I55" s="28"/>
+      <c r="J55" s="28"/>
+      <c r="K55" s="28"/>
+      <c r="L55" s="28"/>
+    </row>
+    <row r="56" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F56" s="42" t="s">
+        <v>127</v>
+      </c>
+      <c r="G56" s="42"/>
+      <c r="H56" s="42"/>
+      <c r="I56" s="42"/>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A57" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="B57" s="25"/>
+      <c r="C57" s="25"/>
+      <c r="D57" s="25"/>
+      <c r="E57" s="25"/>
+      <c r="F57" s="25"/>
+      <c r="I57" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="J57" s="26"/>
+      <c r="K57" s="26"/>
+      <c r="L57" s="26"/>
+      <c r="M57" s="26"/>
+      <c r="N57" s="26"/>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A58" s="29">
+        <v>149</v>
+      </c>
+      <c r="B58" s="29"/>
+      <c r="C58" s="29"/>
+      <c r="D58" s="29"/>
+      <c r="E58" s="29"/>
+      <c r="F58" s="29"/>
+      <c r="I58" s="30">
+        <v>41</v>
+      </c>
+      <c r="J58" s="30"/>
+      <c r="K58" s="30"/>
+      <c r="L58" s="30"/>
+      <c r="M58" s="30"/>
+      <c r="N58" s="30"/>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A59" s="29"/>
+      <c r="B59" s="29"/>
+      <c r="C59" s="29"/>
+      <c r="D59" s="29"/>
+      <c r="E59" s="29"/>
+      <c r="F59" s="29"/>
+      <c r="I59" s="30"/>
+      <c r="J59" s="30"/>
+      <c r="K59" s="30"/>
+      <c r="L59" s="30"/>
+      <c r="M59" s="30"/>
+      <c r="N59" s="30"/>
+    </row>
+    <row r="61" ht="38" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A61" s="43" t="s">
+        <v>130</v>
+      </c>
+      <c r="B61" s="43"/>
+      <c r="C61" s="43"/>
+      <c r="D61" s="43"/>
+      <c r="E61" s="43"/>
+      <c r="F61" s="43"/>
+      <c r="G61" s="43"/>
+      <c r="H61" s="43"/>
+      <c r="I61" s="43"/>
+      <c r="J61" s="43"/>
+      <c r="K61" s="43"/>
+      <c r="L61" s="43"/>
+      <c r="M61" s="43"/>
+      <c r="N61" s="43"/>
     </row>
   </sheetData>
   <autoFilter ref="A6:B6"/>
-  <mergeCells count="2">
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
+  <mergeCells count="39">
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="B18:N18"/>
+    <mergeCell ref="A21:N21"/>
+    <mergeCell ref="A22:N22"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:N24"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="D25:F26"/>
+    <mergeCell ref="G25:I26"/>
+    <mergeCell ref="J25:N26"/>
+    <mergeCell ref="A28:N28"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A41:N41"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A51:N51"/>
+    <mergeCell ref="C53:L53"/>
+    <mergeCell ref="C54:L55"/>
+    <mergeCell ref="F56:I56"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="I57:N57"/>
+    <mergeCell ref="A58:F59"/>
+    <mergeCell ref="I58:N59"/>
+    <mergeCell ref="A61:N61"/>
   </mergeCells>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: count every CRM client as a friendly baseline
</commit_message>
<xml_diff>
--- a/reports/דו״ח-קשרים-אחדות-יהודית.xlsx
+++ b/reports/דו״ח-קשרים-אחדות-יהודית.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="130">
   <si>
     <t>דו״ח קשרים — אחדות יהודית</t>
   </si>
@@ -331,7 +331,7 @@
     <t>משפט סיכום</t>
   </si>
   <si>
-    <t>בכל ההיסטוריה הקיימת במערכת בוצעו בסך הכול 797 קשרים: 438 קשרים תורניים, 274 קשרים ידידותיים, 276 קשרים פרונטליים, 36 קשרי וידאו, 479 קשרים טלפוניים ו־6 אירוחי שבת.</t>
+    <t>בכל ההיסטוריה הקיימת במערכת בוצעו בסך הכול 855 קשרים: 438 קשרים תורניים, 332 קשרים ידידותיים, 276 קשרים פרונטליים, 36 קשרי וידאו, 479 קשרים טלפוניים ו־6 אירוחי שבת.</t>
   </si>
   <si>
     <t>תמונת מצב מנהלים</t>
@@ -367,18 +367,15 @@
     <t>תורני · סוגים נוספים</t>
   </si>
   <si>
-    <t>ידידותי · סוגים נוספים</t>
-  </si>
-  <si>
-    <t>סוגים נוספים כוללים אירוח שבת וכל סוג קשר שאינו פרונטלי, וידאו או טלפוני.</t>
+    <t>ידידותי · קשר בסיס / סוגים נוספים</t>
+  </si>
+  <si>
+    <t>קשר בסיס ידידותי נספר ללקוח ללא קשר מתועד; סוגים נוספים כוללים אירוח שבת וכל סוג שאינו פרונטלי, וידאו או טלפוני.</t>
   </si>
   <si>
     <t>התפלגות לקוחות לפי מספר קשרים</t>
   </si>
   <si>
-    <t>0 קשרים</t>
-  </si>
-  <si>
     <t>קשר אחד</t>
   </si>
   <si>
@@ -409,7 +406,7 @@
     <t>קשר אישי ידידותי</t>
   </si>
   <si>
-    <t>המאגר הכללי הוא נתון הנהלה משוער. הקבוצות האישיות מחושבות מנתוני ה־CRM; קשר תורני אחד לפחות מסווג לקוח כ״אישי תורני״. 9 לקוחות פעילים טרם סווגו כאישי תורני או ידידותי.</t>
+    <t>המאגר הכללי הוא נתון הנהלה משוער. כל לקוח מתועד נחשב לפחות לקשר בסיס ידידותי; קשר תורני אחד לפחות מסווג אותו כ״אישי תורני״.</t>
   </si>
 </sst>
 </file>
@@ -1212,13 +1209,13 @@
         <v>26</v>
       </c>
       <c r="C7" s="12">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D7" s="12">
         <v>16</v>
       </c>
       <c r="E7" s="12">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F7" s="12">
         <v>45</v>
@@ -1236,10 +1233,10 @@
         <v>1018</v>
       </c>
       <c r="K7" s="13">
-        <v>3.769230769230769</v>
+        <v>3.8846153846153846</v>
       </c>
       <c r="L7" s="13">
-        <v>10.387755102040817</v>
+        <v>10.07920792079208</v>
       </c>
     </row>
     <row r="8" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1364,13 +1361,13 @@
         <v>23</v>
       </c>
       <c r="C11" s="12">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D11" s="12">
         <v>32</v>
       </c>
       <c r="E11" s="12">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F11" s="12">
         <v>6</v>
@@ -1388,10 +1385,10 @@
         <v>377</v>
       </c>
       <c r="K11" s="13">
-        <v>2.608695652173913</v>
+        <v>2.8260869565217392</v>
       </c>
       <c r="L11" s="13">
-        <v>6.283333333333333</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="12" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1516,13 +1513,13 @@
         <v>9</v>
       </c>
       <c r="C15" s="12">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D15" s="12">
         <v>29</v>
       </c>
       <c r="E15" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" s="12">
         <v>14</v>
@@ -1540,10 +1537,10 @@
         <v>469</v>
       </c>
       <c r="K15" s="13">
-        <v>3.3333333333333335</v>
+        <v>3.4444444444444446</v>
       </c>
       <c r="L15" s="13">
-        <v>15.633333333333333</v>
+        <v>15.129032258064516</v>
       </c>
     </row>
     <row r="16" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1627,16 +1624,16 @@
         <v>27</v>
       </c>
       <c r="B18" s="12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C18" s="12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D18" s="12">
         <v>0</v>
       </c>
       <c r="E18" s="12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F18" s="12">
         <v>0</v>
@@ -1654,7 +1651,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" s="13">
         <v>0</v>
@@ -1744,13 +1741,13 @@
         <v>4</v>
       </c>
       <c r="C21" s="12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D21" s="12">
         <v>0</v>
       </c>
       <c r="E21" s="12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F21" s="12">
         <v>1</v>
@@ -1768,10 +1765,10 @@
         <v>16</v>
       </c>
       <c r="K21" s="13">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="L21" s="13">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1782,13 +1779,13 @@
         <v>14</v>
       </c>
       <c r="C22" s="12">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D22" s="12">
         <v>4</v>
       </c>
       <c r="E22" s="12">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F22" s="12">
         <v>8</v>
@@ -1806,10 +1803,10 @@
         <v>512</v>
       </c>
       <c r="K22" s="13">
-        <v>2.2857142857142856</v>
+        <v>2.5</v>
       </c>
       <c r="L22" s="13">
-        <v>16</v>
+        <v>14.628571428571428</v>
       </c>
     </row>
     <row r="23" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1820,13 +1817,13 @@
         <v>14</v>
       </c>
       <c r="C23" s="12">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D23" s="12">
         <v>32</v>
       </c>
       <c r="E23" s="12">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F23" s="12">
         <v>11</v>
@@ -1844,10 +1841,10 @@
         <v>547</v>
       </c>
       <c r="K23" s="13">
-        <v>2.7857142857142856</v>
+        <v>3</v>
       </c>
       <c r="L23" s="13">
-        <v>14.025641025641026</v>
+        <v>13.023809523809524</v>
       </c>
     </row>
     <row r="24" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1934,13 +1931,13 @@
         <v>21</v>
       </c>
       <c r="C26" s="12">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D26" s="12">
         <v>41</v>
       </c>
       <c r="E26" s="12">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F26" s="12">
         <v>11</v>
@@ -1958,10 +1955,10 @@
         <v>709</v>
       </c>
       <c r="K26" s="13">
-        <v>2.142857142857143</v>
+        <v>2.619047619047619</v>
       </c>
       <c r="L26" s="13">
-        <v>15.755555555555556</v>
+        <v>12.89090909090909</v>
       </c>
     </row>
     <row r="27" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -2200,13 +2197,13 @@
         <v>12</v>
       </c>
       <c r="C33" s="12">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D33" s="12">
         <v>29</v>
       </c>
       <c r="E33" s="12">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F33" s="12">
         <v>12</v>
@@ -2224,10 +2221,10 @@
         <v>512</v>
       </c>
       <c r="K33" s="13">
-        <v>2.6666666666666665</v>
+        <v>3</v>
       </c>
       <c r="L33" s="13">
-        <v>16</v>
+        <v>14.222222222222221</v>
       </c>
     </row>
     <row r="34" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -2276,13 +2273,13 @@
         <v>10</v>
       </c>
       <c r="C35" s="12">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D35" s="12">
         <v>25</v>
       </c>
       <c r="E35" s="12">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F35" s="12">
         <v>31</v>
@@ -2300,10 +2297,10 @@
         <v>1522</v>
       </c>
       <c r="K35" s="13">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="L35" s="13">
-        <v>20.293333333333333</v>
+        <v>19.766233766233768</v>
       </c>
     </row>
     <row r="36" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -2314,13 +2311,13 @@
         <v>3</v>
       </c>
       <c r="C36" s="12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D36" s="12">
         <v>4</v>
       </c>
       <c r="E36" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36" s="12">
         <v>4</v>
@@ -2338,10 +2335,10 @@
         <v>64</v>
       </c>
       <c r="K36" s="13">
-        <v>1.3333333333333333</v>
+        <v>1.6666666666666667</v>
       </c>
       <c r="L36" s="13">
-        <v>16</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="37" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -2352,13 +2349,13 @@
         <v>31</v>
       </c>
       <c r="C37" s="12">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="D37" s="12">
         <v>22</v>
       </c>
       <c r="E37" s="12">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="F37" s="12">
         <v>22</v>
@@ -2376,10 +2373,10 @@
         <v>423</v>
       </c>
       <c r="K37" s="13">
-        <v>1.096774193548387</v>
+        <v>1.7419354838709677</v>
       </c>
       <c r="L37" s="13">
-        <v>12.441176470588236</v>
+        <v>7.833333333333333</v>
       </c>
     </row>
     <row r="38" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -2425,16 +2422,16 @@
         <v>48</v>
       </c>
       <c r="B39" s="15">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C39" s="15">
-        <v>797</v>
+        <v>855</v>
       </c>
       <c r="D39" s="15">
         <v>438</v>
       </c>
       <c r="E39" s="15">
-        <v>274</v>
+        <v>332</v>
       </c>
       <c r="F39" s="15">
         <v>276</v>
@@ -2452,10 +2449,10 @@
         <v>10638</v>
       </c>
       <c r="K39" s="16">
-        <v>3.1377952755905514</v>
+        <v>3.3268482490272375</v>
       </c>
       <c r="L39" s="16">
-        <v>13.347553324968633</v>
+        <v>12.442105263157895</v>
       </c>
     </row>
   </sheetData>
@@ -4590,7 +4587,7 @@
         <v>102</v>
       </c>
       <c r="B7" s="21">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4598,7 +4595,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="21">
-        <v>797</v>
+        <v>855</v>
       </c>
     </row>
     <row r="9" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4614,7 +4611,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="21">
-        <v>274</v>
+        <v>332</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4662,7 +4659,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="21">
-        <v>3.1377952755905514</v>
+        <v>3.3268482490272375</v>
       </c>
     </row>
     <row r="17" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4670,7 +4667,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="21">
-        <v>13.347553324968633</v>
+        <v>12.442105263157895</v>
       </c>
     </row>
     <row r="18" ht="54" customHeight="1" spans="1:14" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -4755,7 +4752,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="28">
-        <v>199</v>
+        <v>257</v>
       </c>
       <c r="B25" s="28"/>
       <c r="C25" s="28"/>
@@ -4765,12 +4762,12 @@
       <c r="E25" s="29"/>
       <c r="F25" s="29"/>
       <c r="G25" s="30">
-        <v>274</v>
+        <v>332</v>
       </c>
       <c r="H25" s="30"/>
       <c r="I25" s="30"/>
       <c r="J25" s="31">
-        <v>797</v>
+        <v>855</v>
       </c>
       <c r="K25" s="31"/>
       <c r="L25" s="31"/>
@@ -4958,10 +4955,10 @@
       <c r="B37" s="33"/>
       <c r="C37" s="33"/>
       <c r="D37" s="37">
-        <v>0</v>
-      </c>
-      <c r="E37" s="36"/>
-      <c r="F37" s="36"/>
+        <v>58</v>
+      </c>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
       <c r="G37" s="36"/>
       <c r="H37" s="36"/>
       <c r="I37" s="36"/>
@@ -5014,7 +5011,7 @@
       <c r="B43" s="33"/>
       <c r="C43" s="33"/>
       <c r="D43" s="40">
-        <v>55</v>
+        <v>111</v>
       </c>
       <c r="E43" s="41"/>
       <c r="F43" s="41"/>
@@ -5034,18 +5031,18 @@
       <c r="B44" s="33"/>
       <c r="C44" s="33"/>
       <c r="D44" s="40">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E44" s="41"/>
       <c r="F44" s="41"/>
       <c r="G44" s="41"/>
-      <c r="H44" s="41"/>
-      <c r="I44" s="41"/>
-      <c r="J44" s="41"/>
-      <c r="K44" s="41"/>
-      <c r="L44" s="41"/>
-      <c r="M44" s="41"/>
-      <c r="N44" s="41"/>
+      <c r="H44" s="36"/>
+      <c r="I44" s="36"/>
+      <c r="J44" s="36"/>
+      <c r="K44" s="36"/>
+      <c r="L44" s="36"/>
+      <c r="M44" s="36"/>
+      <c r="N44" s="36"/>
     </row>
     <row r="45" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="33" t="s">
@@ -5054,14 +5051,14 @@
       <c r="B45" s="33"/>
       <c r="C45" s="33"/>
       <c r="D45" s="40">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="E45" s="41"/>
       <c r="F45" s="41"/>
       <c r="G45" s="41"/>
       <c r="H45" s="41"/>
-      <c r="I45" s="41"/>
-      <c r="J45" s="41"/>
+      <c r="I45" s="36"/>
+      <c r="J45" s="36"/>
       <c r="K45" s="36"/>
       <c r="L45" s="36"/>
       <c r="M45" s="36"/>
@@ -5074,17 +5071,17 @@
       <c r="B46" s="33"/>
       <c r="C46" s="33"/>
       <c r="D46" s="40">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E46" s="41"/>
       <c r="F46" s="41"/>
       <c r="G46" s="41"/>
       <c r="H46" s="41"/>
-      <c r="I46" s="41"/>
-      <c r="J46" s="41"/>
-      <c r="K46" s="41"/>
-      <c r="L46" s="41"/>
-      <c r="M46" s="41"/>
+      <c r="I46" s="36"/>
+      <c r="J46" s="36"/>
+      <c r="K46" s="36"/>
+      <c r="L46" s="36"/>
+      <c r="M46" s="36"/>
       <c r="N46" s="36"/>
     </row>
     <row r="47" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -5094,42 +5091,22 @@
       <c r="B47" s="33"/>
       <c r="C47" s="33"/>
       <c r="D47" s="40">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E47" s="41"/>
-      <c r="F47" s="41"/>
-      <c r="G47" s="41"/>
-      <c r="H47" s="41"/>
-      <c r="I47" s="41"/>
-      <c r="J47" s="41"/>
-      <c r="K47" s="41"/>
-      <c r="L47" s="41"/>
-      <c r="M47" s="41"/>
+      <c r="F47" s="36"/>
+      <c r="G47" s="36"/>
+      <c r="H47" s="36"/>
+      <c r="I47" s="36"/>
+      <c r="J47" s="36"/>
+      <c r="K47" s="36"/>
+      <c r="L47" s="36"/>
+      <c r="M47" s="36"/>
       <c r="N47" s="36"/>
-    </row>
-    <row r="48" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A48" s="33" t="s">
-        <v>124</v>
-      </c>
-      <c r="B48" s="33"/>
-      <c r="C48" s="33"/>
-      <c r="D48" s="40">
-        <v>16</v>
-      </c>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="36"/>
-      <c r="I48" s="36"/>
-      <c r="J48" s="36"/>
-      <c r="K48" s="36"/>
-      <c r="L48" s="36"/>
-      <c r="M48" s="36"/>
-      <c r="N48" s="36"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="22" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B51" s="22"/>
       <c r="C51" s="22"/>
@@ -5147,7 +5124,7 @@
     </row>
     <row r="53" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C53" s="24" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D53" s="24"/>
       <c r="E53" s="24"/>
@@ -5187,7 +5164,7 @@
     </row>
     <row r="56" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F56" s="42" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G56" s="42"/>
       <c r="H56" s="42"/>
@@ -5195,7 +5172,7 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="25" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B57" s="25"/>
       <c r="C57" s="25"/>
@@ -5203,7 +5180,7 @@
       <c r="E57" s="25"/>
       <c r="F57" s="25"/>
       <c r="I57" s="26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J57" s="26"/>
       <c r="K57" s="26"/>
@@ -5221,7 +5198,7 @@
       <c r="E58" s="29"/>
       <c r="F58" s="29"/>
       <c r="I58" s="30">
-        <v>41</v>
+        <v>108</v>
       </c>
       <c r="J58" s="30"/>
       <c r="K58" s="30"/>
@@ -5245,7 +5222,7 @@
     </row>
     <row r="61" ht="38" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="43" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B61" s="43"/>
       <c r="C61" s="43"/>
@@ -5263,7 +5240,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A6:B6"/>
-  <mergeCells count="39">
+  <mergeCells count="38">
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="B18:N18"/>
@@ -5293,7 +5270,6 @@
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A46:C46"/>
     <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A48:C48"/>
     <mergeCell ref="A51:N51"/>
     <mergeCell ref="C53:L53"/>
     <mergeCell ref="C54:L55"/>

</xml_diff>